<commit_message>
nieuwe concessiecodes en verbetering 2023
</commit_message>
<xml_diff>
--- a/Stationscodes.xlsx
+++ b/Stationscodes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Mobiliteit-projecten\OV_Oost_reizigers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F42C131-B685-4503-A372-7231DCA7C9C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{700BCF67-E286-4B84-8CC7-8835806DFA03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1515" yWindow="1515" windowWidth="21600" windowHeight="11265" xr2:uid="{0CE0F5B6-8556-47E6-9FDF-B5EC4AD1392A}"/>
+    <workbookView xWindow="-24120" yWindow="2490" windowWidth="24240" windowHeight="13140" xr2:uid="{0CE0F5B6-8556-47E6-9FDF-B5EC4AD1392A}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="49">
   <si>
     <t>HNR</t>
   </si>
@@ -160,6 +160,30 @@
   </si>
   <si>
     <t>Gronau</t>
+  </si>
+  <si>
+    <t>Barneveld Zuid</t>
+  </si>
+  <si>
+    <t>Ede-Wageningen</t>
+  </si>
+  <si>
+    <t>Ede Centrum</t>
+  </si>
+  <si>
+    <t>Lunteren</t>
+  </si>
+  <si>
+    <t>Hoevelaken</t>
+  </si>
+  <si>
+    <t>Amersfoort Centraal</t>
+  </si>
+  <si>
+    <t>Barneveld Centrum</t>
+  </si>
+  <si>
+    <t>Barneveld Noord</t>
   </si>
 </sst>
 </file>
@@ -249,9 +273,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Kantoorthema">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Thema">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -289,7 +313,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -395,7 +419,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -537,7 +561,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -545,7 +569,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF6F9838-ED03-4852-9CD1-56A337459079}">
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G64"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.5703125" customWidth="1"/>
@@ -1064,6 +1088,70 @@
         <v>398</v>
       </c>
     </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>41</v>
+      </c>
+      <c r="B57">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>42</v>
+      </c>
+      <c r="B58">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>43</v>
+      </c>
+      <c r="B59">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>44</v>
+      </c>
+      <c r="B60">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>45</v>
+      </c>
+      <c r="B61">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>46</v>
+      </c>
+      <c r="B62">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>47</v>
+      </c>
+      <c r="B63">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>48</v>
+      </c>
+      <c r="B64">
+        <v>92</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="D40:G55">
     <sortCondition ref="D40:D55"/>

</xml_diff>